<commit_message>
Ajustes na tela de cadastro, lógica de perfis PF/PJ, correção de duplicidade e natureza das transações
</commit_message>
<xml_diff>
--- a/modelo_importacao.xlsx
+++ b/modelo_importacao.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\elien\OneDrive\Documentos\app-financeiro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{20260222-B3C1-49AB-A630-16628A9EA816}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4EF97C87-354D-4A3B-B9F4-2C4F2C0C9928}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Importacao" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="19">
   <si>
     <t>Data</t>
   </si>
@@ -31,22 +31,52 @@
     <t>Valor</t>
   </si>
   <si>
-    <t>01/01/2026</t>
-  </si>
-  <si>
-    <t>Venda de Software</t>
-  </si>
-  <si>
-    <t>05/01/2026</t>
-  </si>
-  <si>
-    <t>Aluguel Escritorio</t>
-  </si>
-  <si>
-    <t>10/01/2026</t>
-  </si>
-  <si>
-    <t>Serviços Prestados</t>
+    <t>Dinheiro retirado Emergências</t>
+  </si>
+  <si>
+    <t>Pagamento com QR Pix 99 FOOD LTDA.</t>
+  </si>
+  <si>
+    <t>Dinheiro reservado Emergências</t>
+  </si>
+  <si>
+    <t>Pagamento com QR Pix SDB COMERCIO DE ALIMENTOS LTDA</t>
+  </si>
+  <si>
+    <t>Pagamento com QR Pix IFOOD.COM AGENCIA DE RESTAURANTES ONLINE S.A.</t>
+  </si>
+  <si>
+    <t>Pagamento de conta Banco Santander (Brasil) S. A.</t>
+  </si>
+  <si>
+    <t>Pix enviado Nubia Ximenes Aragao</t>
+  </si>
+  <si>
+    <t>Pix recebido 58.109.673 VINICIUS COSTA NUNES</t>
+  </si>
+  <si>
+    <t>Pagamento com QR Pix Gustavo Costa Nunes</t>
+  </si>
+  <si>
+    <t>Pix recebido CYBER ALLIANCE IT T. DA I. LTDA</t>
+  </si>
+  <si>
+    <t>Pix enviado Elienay Costa Silva</t>
+  </si>
+  <si>
+    <t>Pagamento com QR Pix RIO GRANDE COMERCIO DE CARNES LTDA</t>
+  </si>
+  <si>
+    <t>Pagamento com QR Pix MATEUS SUPERMERCADOS S A</t>
+  </si>
+  <si>
+    <t>Pagamento com QR Pix KREDIT PAGAMENTOS SA</t>
+  </si>
+  <si>
+    <t>Pix enviado Thais Do Nascimento De Morais</t>
+  </si>
+  <si>
+    <t>Reembolso de transferência enviada 99 FOOD LTDA.</t>
   </si>
 </sst>
 </file>
@@ -82,9 +112,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="4" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -424,10 +455,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C4"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:C34"/>
+  <sheetFormatPr defaultRowHeight="15.6" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="84.3984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="8.5" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -438,43 +474,373 @@
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
-        <v>3</v>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A2" s="2">
+        <v>46082</v>
       </c>
       <c r="B2" t="s">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="C2" s="1">
-        <v>1500</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A3" t="s">
-        <v>5</v>
+        <v>70</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A3" s="2">
+        <v>46082</v>
       </c>
       <c r="B3" t="s">
         <v>6</v>
       </c>
       <c r="C3" s="1">
-        <v>-2500</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" t="s">
+        <v>-70.06</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A4" s="2">
+        <v>46084</v>
+      </c>
+      <c r="B4" t="s">
         <v>7</v>
       </c>
-      <c r="B4" t="s">
+      <c r="C4" s="1">
+        <v>-16.989999999999998</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="2">
+        <v>46084</v>
+      </c>
+      <c r="B5" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="1">
+        <v>931.2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="2">
+        <v>46084</v>
+      </c>
+      <c r="B6" t="s">
         <v>8</v>
       </c>
-      <c r="C4" s="1">
-        <v>3000</v>
+      <c r="C6" s="1">
+        <v>-908.65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A7" s="2">
+        <v>46084</v>
+      </c>
+      <c r="B7" t="s">
+        <v>9</v>
+      </c>
+      <c r="C7" s="1">
+        <v>-7.5</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A8" s="2">
+        <v>46085</v>
+      </c>
+      <c r="B8" t="s">
+        <v>10</v>
+      </c>
+      <c r="C8" s="1">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A9" s="2">
+        <v>46086</v>
+      </c>
+      <c r="B9" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="1">
+        <v>-5000</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A10" s="2">
+        <v>46087</v>
+      </c>
+      <c r="B10" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="1">
+        <v>-20</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A11" s="2">
+        <v>46088</v>
+      </c>
+      <c r="B11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11" s="1">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A12" s="2">
+        <v>46088</v>
+      </c>
+      <c r="B12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" s="1">
+        <v>-500</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A13" s="2">
+        <v>46094</v>
+      </c>
+      <c r="B13" t="s">
+        <v>12</v>
+      </c>
+      <c r="C13" s="1">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A14" s="2">
+        <v>46094</v>
+      </c>
+      <c r="B14" t="s">
+        <v>5</v>
+      </c>
+      <c r="C14" s="1">
+        <v>-500</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A15" s="2">
+        <v>46094</v>
+      </c>
+      <c r="B15" t="s">
+        <v>13</v>
+      </c>
+      <c r="C15" s="1">
+        <v>-2000</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A16" s="2">
+        <v>46105</v>
+      </c>
+      <c r="B16" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16" s="1">
+        <v>100.36</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="2">
+        <v>46105</v>
+      </c>
+      <c r="B17" t="s">
+        <v>14</v>
+      </c>
+      <c r="C17" s="1">
+        <v>-100.36</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="2">
+        <v>46105</v>
+      </c>
+      <c r="B18" t="s">
+        <v>3</v>
+      </c>
+      <c r="C18" s="1">
+        <v>35.75</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A19" s="2">
+        <v>46105</v>
+      </c>
+      <c r="B19" t="s">
+        <v>15</v>
+      </c>
+      <c r="C19" s="1">
+        <v>-35.75</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A20" s="2">
+        <v>46105</v>
+      </c>
+      <c r="B20" t="s">
+        <v>3</v>
+      </c>
+      <c r="C20" s="1">
+        <v>137.94999999999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A21" s="2">
+        <v>46105</v>
+      </c>
+      <c r="B21" t="s">
+        <v>15</v>
+      </c>
+      <c r="C21" s="1">
+        <v>-137.94999999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A22" s="2">
+        <v>46108</v>
+      </c>
+      <c r="B22" t="s">
+        <v>3</v>
+      </c>
+      <c r="C22" s="1">
+        <v>24.9</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A23" s="2">
+        <v>46108</v>
+      </c>
+      <c r="B23" t="s">
+        <v>16</v>
+      </c>
+      <c r="C23" s="1">
+        <v>-24.9</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A24" s="2">
+        <v>46108</v>
+      </c>
+      <c r="B24" t="s">
+        <v>3</v>
+      </c>
+      <c r="C24" s="1">
+        <v>18.27</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A25" s="2">
+        <v>46108</v>
+      </c>
+      <c r="B25" t="s">
+        <v>4</v>
+      </c>
+      <c r="C25" s="1">
+        <v>-18.27</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A26" s="2">
+        <v>46109</v>
+      </c>
+      <c r="B26" t="s">
+        <v>10</v>
+      </c>
+      <c r="C26" s="1">
+        <v>5000</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A27" s="2">
+        <v>46109</v>
+      </c>
+      <c r="B27" t="s">
+        <v>5</v>
+      </c>
+      <c r="C27" s="1">
+        <v>-5000</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A28" s="2">
+        <v>46110</v>
+      </c>
+      <c r="B28" t="s">
+        <v>3</v>
+      </c>
+      <c r="C28" s="1">
+        <v>4000</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A29" s="2">
+        <v>46110</v>
+      </c>
+      <c r="B29" t="s">
+        <v>17</v>
+      </c>
+      <c r="C29" s="1">
+        <v>-4000</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A30" s="2">
+        <v>46111</v>
+      </c>
+      <c r="B30" t="s">
+        <v>3</v>
+      </c>
+      <c r="C30" s="1">
+        <v>18.440000000000001</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A31" s="2">
+        <v>46111</v>
+      </c>
+      <c r="B31" t="s">
+        <v>4</v>
+      </c>
+      <c r="C31" s="1">
+        <v>-18.440000000000001</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A32" s="2">
+        <v>46112</v>
+      </c>
+      <c r="B32" t="s">
+        <v>3</v>
+      </c>
+      <c r="C32" s="1">
+        <v>21.68</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A33" s="2">
+        <v>46112</v>
+      </c>
+      <c r="B33" t="s">
+        <v>4</v>
+      </c>
+      <c r="C33" s="1">
+        <v>-21.68</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A34" s="2">
+        <v>46112</v>
+      </c>
+      <c r="B34" t="s">
+        <v>18</v>
+      </c>
+      <c r="C34" s="1">
+        <v>21.68</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <ignoredErrors>
-    <ignoredError sqref="A1:C1 A4:B4 A2:B2 A3:B3" numberStoredAsText="1"/>
+    <ignoredError sqref="A1:C1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>